<commit_message>
Update DLS journal + dls.json
</commit_message>
<xml_diff>
--- a/data/Журнал_ДЛС.xlsx
+++ b/data/Журнал_ДЛС.xlsx
@@ -7201,7 +7201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H42"/>
+  <dimension ref="A1:H54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -8396,17 +8396,17 @@
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>№ 336-001.001/002.0/17-26 від 24.07.2026</t>
+          <t>№ 335-001.001/002.0/17-26 від 22.07.2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>24.07.2026</t>
+          <t>22.07.2026</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>ПАКЛІТАКСЕЛ АМАКСА, концентрат для розчину для інфузій, 6 мг/мл; по 5 мл, 16,7 мл або 50 мл у флаконі; по 1 флакону в картонній коробці, Серія № AO261002, контроль та випуск серії: АкВіда ГмбХ, Німеччина виробництво in bulk, первинне та вторинне пакування: Самянг Холдінгз Корпорейшн, Республiка Корея виробництво in bulk, первинне пакування, вторинне пакування, контроль серії: АкВіда ГмбХ, Німеччина, Німеччина/ Республiка Корея</t>
+          <t>ЦЕФЕПІМ АНАНТА, порошок для розчину для ін'єкцій по 2 г; 1 або 10 флаконів з порошком в коробці, Серія № всі серії, Ананта Медікеар Лімітед, Індія</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -8417,6 +8417,342 @@
       <c r="F42" s="2" t="inlineStr"/>
       <c r="G42" s="2" t="inlineStr"/>
       <c r="H42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43" ht="40" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>№ 335-001.001/002.0/17-26 від 22.07.2026</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>22.07.2026</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>ЦЕФЕПІМ АНАНТА, порошок для розчину для ін'єкцій по 1 г; 1 або 10 флаконів з порошком в коробці, Серія № всі серії, Ананта Медікеар Лімітед, Індія</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+      <c r="H43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="40" customHeight="1">
+      <c r="A44" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>№ 336-001.001/002.0/17-26 від 24.07.2026</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>24.07.2026</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>ПАКЛІТАКСЕЛ АМАКСА, концентрат для розчину для інфузій, 6 мг/мл; по 5 мл, 16,7 мл або 50 мл у флаконі; по 1 флакону в картонній коробці, Серія № AO261002, контроль та випуск серії: АкВіда ГмбХ, Німеччина виробництво in bulk, первинне та вторинне пакування: Самянг Холдінгз Корпорейшн, Республiка Корея виробництво in bulk, первинне пакування, вторинне пакування, контроль серії: АкВіда ГмбХ, Німеччина, Німеччина/ Республiка Корея</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+      <c r="H44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45" ht="40" customHeight="1">
+      <c r="A45" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>№ 337-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>ЛОПЕРАМІД, таблетки по 2 мг по 10 таблеток у блістері; по 2 блістери в пачці, Серія № 011188, ТОВ "МАРІФАРМ", Словенія</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+      <c r="H45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46" ht="40" customHeight="1">
+      <c r="A46" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>№ 339-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>ГАБАНА®, капсули по 300 мг, по 10 капсул у блістері; по 2 блістери в пачці, Серія № 011523, ТОВ «МАРІФАРМ», Словенія</t>
+        </is>
+      </c>
+      <c r="E46" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+      <c r="H46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47" ht="40" customHeight="1">
+      <c r="A47" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>№ 339-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>ГАБАНА®, капсули по 300 мг, по 10 капсул у блістері; по 2 блістери в пачці, Серія № 011520, ТОВ «МАРІФАРМ», Словенія</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+      <c r="H47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48" ht="40" customHeight="1">
+      <c r="A48" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>№ 339-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D48" s="2" t="inlineStr">
+        <is>
+          <t>ГАБАНА®, капсули по 300 мг, по 10 капсул у блістері; по 2 блістери в пачці, Серія № 011502, ТОВ «МАРІФАРМ», Словенія</t>
+        </is>
+      </c>
+      <c r="E48" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+      <c r="H48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>№ 342-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="inlineStr">
+        <is>
+          <t>САЛІЦИЛОВА МАЗЬ, мазь 10 % по 25 г у тубі ламінатній в пачці, Серія № 010124, ПрАТ Фармацевтична фабрика "Віола", Україна</t>
+        </is>
+      </c>
+      <c r="E49" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+      <c r="H49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50" ht="40" customHeight="1">
+      <c r="A50" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>№ 342-001.001/002.0/17-26 від 27.07.2026</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>27.07.2026</t>
+        </is>
+      </c>
+      <c r="D50" s="2" t="inlineStr">
+        <is>
+          <t>САЛІЦИЛОВА МАЗЬ, мазь 10% по 25 г у тубі ламінатній в пачці, Серія № 090824, ПрАТ Фармацевтична фабрика "Віола", Україна</t>
+        </is>
+      </c>
+      <c r="E50" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+      <c r="H50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51" ht="40" customHeight="1">
+      <c r="A51" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>№ 343-001.001/002.0/17-26 від 28.07.2026</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="D51" s="2" t="inlineStr">
+        <is>
+          <t>ЕМЛА, крем по 30 г у тубі; по 1 тубі у картонній коробці, Серія № 100272, Ресіфарм Карлскога АБ, Австрія</t>
+        </is>
+      </c>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+      <c r="H51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52" ht="40" customHeight="1">
+      <c r="A52" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>№ 344-001.001/002.0/17-26 від 28.07.2026</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>VALAMOR (ribociclib) 200 mg, таблетки № 63, Серія № A0213K, Novartis Sagl?k, G?da ve Tar?m Urunleri San. ve Tic. A.S., -</t>
+        </is>
+      </c>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+      <c r="H52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53" ht="40" customHeight="1">
+      <c r="A53" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>№ 345-001.001/002.0/17-26 від 28.07.2026</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="D53" s="2" t="inlineStr">
+        <is>
+          <t>ФІБРИНАЗА-20, таблетки, вкриті оболонкою, кишковорозчинні по 20 мг; по 10 таблеток у блістері; по 3 блістери у картонній пачці, Серія № EBK25010B1, EBK25011B1, EBK25012B1, EBK26004B1, EBK26005B1, EBK26007B1, Евертоджен Лайф Саєнсиз  Лімітед, Індія</t>
+        </is>
+      </c>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+      <c r="H53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54" ht="40" customHeight="1">
+      <c r="A54" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>№ 345-001.001/002.0/17-26 від 28.07.2026</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>28.07.2026</t>
+        </is>
+      </c>
+      <c r="D54" s="2" t="inlineStr">
+        <is>
+          <t>ФІБРИНАЗА-10, таблетки, вкриті оболонкою, кишковорозчинні по 10 мг, по 10 таблеток у блістері; по 3 блістери у картонній пачці, Серія № ESI25011B1, ESI25012B1, ESI26002B1, ESI26003B1, Евертоджен Лайф Саєнсиз Лімітед, Індія</t>
+        </is>
+      </c>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>відсутній</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+      <c r="H54" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>